<commit_message>
Add address column to employee sheet from address sheet
- Matched addresses by name column
- davy: sydney
- flora: meoborne

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/excel-guy-test2.xlsx
+++ b/excel-guy-test2.xlsx
@@ -1,87 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/M017224/OnDisk/Public/ai-test/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A72F86B2-4371-0F48-83EE-B7228868CB06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3260" yWindow="2260" windowWidth="28040" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3260" yWindow="2260" windowWidth="28040" windowHeight="17180" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="employee" sheetId="1" r:id="rId1"/>
-    <sheet name="address" sheetId="2" r:id="rId2"/>
+    <sheet name="employee" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="address" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
-  <si>
-    <t xml:space="preserve">name </t>
-  </si>
-  <si>
-    <t>hours worked</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rate </t>
-  </si>
-  <si>
-    <t>total</t>
-  </si>
-  <si>
-    <t>super</t>
-  </si>
-  <si>
-    <t>davy</t>
-  </si>
-  <si>
-    <t>flora</t>
-  </si>
-  <si>
-    <t>address</t>
-  </si>
-  <si>
-    <t>sydney</t>
-  </si>
-  <si>
-    <t>meoborne</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -100,21 +47,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -434,110 +440,164 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:F4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:G10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col width="13.83203125" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" t="s">
-        <v>4</v>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name </t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>hours worked</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rate </t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>super</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>address</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3">
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>davy</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>40</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>28</v>
       </c>
       <c r="E3">
         <f>C3*D3</f>
-        <v>1120</v>
+        <v/>
       </c>
       <c r="F3">
         <f>E3*0.1</f>
-        <v>112</v>
+        <v/>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>sydney</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4">
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>flora</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>35</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>35</v>
       </c>
       <c r="E4">
         <f>C4*D4</f>
-        <v>1225</v>
+        <v/>
       </c>
       <c r="F4">
         <f>E4*0.1</f>
-        <v>122.5</v>
+        <v/>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>meoborne</t>
+        </is>
       </c>
     </row>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1EBE9A7-286C-4A4D-A676-6548FE26B5FD}">
-  <dimension ref="B3:C5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A3:C10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name </t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>address</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>davy</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>sydney</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>flora</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>meoborne</t>
+        </is>
       </c>
     </row>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{cccd100a-077b-4351-b7ea-99b99562cb12}" enabled="1" method="Privileged" siteId="{f06fa858-824b-4a85-aacb-f372cfdc282e}" contentBits="0" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>